<commit_message>
Updated TestCase Excel Sheet
</commit_message>
<xml_diff>
--- a/src/Tariq/TestCasesExcelSheet/TestCases.xlsx
+++ b/src/Tariq/TestCasesExcelSheet/TestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tariq\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1619BD48-3E58-4FB2-A02E-709253A7ECAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE8FFCB5-654B-4513-BEE0-6B248F44DEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{FBFEE464-4A34-449A-B708-FC3517E0BA7B}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="197">
   <si>
     <t>Test Scenario</t>
   </si>
@@ -441,12 +441,463 @@
   <si>
     <t>BUG_003</t>
   </si>
+  <si>
+    <t>Verify Home Page Carousel Functionality</t>
+  </si>
+  <si>
+    <t>Verify the carousel is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>TC_010</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Observe the home page carousel.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>The carousel slide should be displayed successfully with the correct image and content.</t>
+  </si>
+  <si>
+    <t>The carousel was displayed successfully on the home page with the correct image and content.</t>
+  </si>
+  <si>
+    <t>Verify the total number of carousel slide displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Observe the home page carousel.
+4. Click the Next (&gt;) button.</t>
+  </si>
+  <si>
+    <t>6 carousel slide should be displayed successfully with the correct image and content.</t>
+  </si>
+  <si>
+    <t>6 carousel was displayed successfully on the home page with the correct image and content.</t>
+  </si>
+  <si>
+    <t>TC_011</t>
+  </si>
+  <si>
+    <t>TC_012</t>
+  </si>
+  <si>
+    <t>Verify clicking on the carousel slide "The Best Online Learning Platform" redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click on the Read More Button on  "The Best Online Learning Platform" carousel slide.</t>
+  </si>
+  <si>
+    <t>TC_013</t>
+  </si>
+  <si>
+    <t>Verify clicking on the carousel slide "Master the basics of software testing" redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Courses Categories page associated with the "The Best Online Learning Platform" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Courses Categories page associated with the "The Best Online Learning Platform" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Manual Testing page associated with the "Master the basics of software testing" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Manual Testing page associated with the "Master the basics of software testing" carousel slide.</t>
+  </si>
+  <si>
+    <t>Verify clicking on the carousel slide "Become an Automation Testing Pro" redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click 2 times Next (&gt;) button.
+4. Click on the Read More Button on  "Become an Automation Testing Pro" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Automation Testing page associated with the "Become an Automation Testing Pro" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Automation Testing page associated with the "Become an Automation Testing Pro" carousel slide.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click 1 time the Next (&gt;) button.
+4. Click on the Read More Button on  "Master the basics of software testing" carousel slide.</t>
+  </si>
+  <si>
+    <t>Verify clicking on the carousel slide "Master API Testing Essentials" redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the API Testing page associated with the "Master API Testing Essentials" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the API Testing page associated with the "Master API Testing Essentials" carousel slide.</t>
+  </si>
+  <si>
+    <t>Verify clicking on the carousel slide "Master Manual, Automation &amp; API" redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click 4 times Next (&gt;) button.
+4. Click on the Read More Button on  "Master Manual, Automation &amp; API" carousel slide.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click 3 times Next (&gt;) button.
+4. Click on the Read More Button on  "Master API Testing Essentials" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Complete Software Testing page associated with the "Master Manual, Automation &amp; API" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Complete Software Testing page associated with the "Master Manual, Automation &amp; API" carousel slide.</t>
+  </si>
+  <si>
+    <t>TC_014</t>
+  </si>
+  <si>
+    <t>TC_015</t>
+  </si>
+  <si>
+    <t>Verify clicking on the carousel slide "Master Java Programming" redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click 5 times Next (&gt;) button.
+4. Click on the Read More Button on  "Master Java Programming" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Core Java page associated with the "Master Java Programming" carousel slide.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Core Java page associated with the "Master Java Programming" carousel slide.</t>
+  </si>
+  <si>
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>TC_017</t>
+  </si>
+  <si>
+    <t>Verify Home Page Information Cards</t>
+  </si>
+  <si>
+    <t>TC_018</t>
+  </si>
+  <si>
+    <t>Verify the "Skilled Instructors" card is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Observe the "Skilled Instructors" card.</t>
+  </si>
+  <si>
+    <t>The "Skilled Instructors" card should be displayed with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <t>The "Skilled Instructors" card was displayed successfully with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <t>TC_019</t>
+  </si>
+  <si>
+    <t>Verify the "Online Classes" card is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Observe the "Online Classes" card.</t>
+  </si>
+  <si>
+    <t>The "Online Classes" card should be displayed with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <t>The "Online Classes" card was displayed successfully with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <t>TC_020</t>
+  </si>
+  <si>
+    <t>TC_021</t>
+  </si>
+  <si>
+    <t>Verify the "Guidance and Support" card is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Observe the "Guidance and Support" card.</t>
+  </si>
+  <si>
+    <t>The "Guidance and Support" card should be displayed with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <t>The "Guidance and Support" card was displayed successfully with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <t>Verify the "Enhanced Learning" card is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Observe the "Enhanced Learning" card.</t>
+  </si>
+  <si>
+    <t>The "Enhanced Learning" card should be displayed with the correct icon, heading, description and colour.</t>
+  </si>
+  <si>
+    <r>
+      <t>The "Enhanced Learning" card was displayed successfully with the correct icon, heading, description but</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> colour was not correct.</t>
+    </r>
+  </si>
+  <si>
+    <t>BUG_004</t>
+  </si>
+  <si>
+    <t>Verify clicking on the "Skilled Instructors" card redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click on "Skilled Instructors" card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Our Team page associated with the "Enhanced Learning" card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Our Team page associated with the "Enhanced Learning" card.</t>
+  </si>
+  <si>
+    <t>TC_022</t>
+  </si>
+  <si>
+    <t>TC_023</t>
+  </si>
+  <si>
+    <t>Verify clicking on the "Online Classes" card redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click on "Online Classes" card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Courses page associated with the "Online Classes" card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Courses page associated with the "Online Classes" card.</t>
+  </si>
+  <si>
+    <t>Verify clicking on the "Guidance and Support" card redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click on "Guidance and Support" card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Contact page associated with the "Guidance and Support" card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Contact page associated with the "Guidance and Support" card.</t>
+  </si>
+  <si>
+    <t>TC_024</t>
+  </si>
+  <si>
+    <t>Verify clicking on the "Enhanced Learning" card redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Click on "Enhanced Learning" card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Complete Software Testing page associated with the "Enhanced Learning" card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Complete Software Testing page associated with the "Enhanced Learning" card.</t>
+  </si>
+  <si>
+    <t>TC_025</t>
+  </si>
+  <si>
+    <t>Verify About Us Section on Home Page</t>
+  </si>
+  <si>
+    <t>TC_026</t>
+  </si>
+  <si>
+    <t>Verify the "About Us" section is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll Down to About Us Section.
+4. Observe the "About Us" section.</t>
+  </si>
+  <si>
+    <t>The "About Us" section should be displayed with the correct image, heading, description, and other related content.</t>
+  </si>
+  <si>
+    <t>The "About Us" section was displayed successfully with the correct image, heading, description, and other related content.</t>
+  </si>
+  <si>
+    <t>TC_027</t>
+  </si>
+  <si>
+    <t>Verify the "Read More" button in the "About Us" section redirects the user to the correct page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll down to the "About Us" section.
+4. Click the "Read More" button.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Courses page associated with the "Read More" button in the "About Us" section.</t>
+  </si>
+  <si>
+    <t>The user was successfully redirected to the Courses page associated with the "Read More" button in the "About Us" section.</t>
+  </si>
+  <si>
+    <t>Verify Course Categories Section on Home Page</t>
+  </si>
+  <si>
+    <t>TC_028</t>
+  </si>
+  <si>
+    <t>Verify the "Course Categories " section is displayed on the home page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll Down to "Course Categories" Section.
+4. Observe the "Course Categories" section.</t>
+  </si>
+  <si>
+    <t>The "Course Categories" section should be displayed with the correct image, heading, description, and other related content.</t>
+  </si>
+  <si>
+    <t>The "Course Categories" section was displayed successfully with the correct image, heading, description, and other related content.</t>
+  </si>
+  <si>
+    <t>TC_029</t>
+  </si>
+  <si>
+    <t>Verify clicking the "Automation Testing" course card redirects the user to the correct course page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll down to the "Course Categories" section.
+4. Observe the Automation Testing course card.
+5. Click the Automation Testing course card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Automation Testing course page, and the page should display 5 courses, matching the count shown on the course card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Automation Testing course page successfully; however, the page displayed only 3 courses, while the course card showed 5 courses.</t>
+  </si>
+  <si>
+    <t>BUG_005</t>
+  </si>
+  <si>
+    <t>TC_030</t>
+  </si>
+  <si>
+    <t>Verify clicking the "Manual Testing" course card redirects the user to the correct course page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll down to the "Course Categories" section.
+4. Observe the Manual Testing course card.
+5. Click the Manual Testing course card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Manual Testing course page, and the page should display 1 course, matching the count shown on the course card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Manual Testing course page successfully; however, the page displayed 3 courses, while the course card showed 1 course.</t>
+  </si>
+  <si>
+    <t>BUG_006</t>
+  </si>
+  <si>
+    <t>TC_031</t>
+  </si>
+  <si>
+    <t>Verify clicking the "Core Java" course card redirects the user to the correct course page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll down to the "Course Categories" section.
+4. Observe the Core Java course card.
+5. Click the Core Java course card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the Core Java course page, and the page should display 1 course, matching the count shown on the course card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Core Java course page successfully; however, the page displayed 3 courses, while the course card showed 1 course.</t>
+  </si>
+  <si>
+    <t>BUG_007</t>
+  </si>
+  <si>
+    <t>Verify clicking the "API Testing" course card redirects the user to the correct course page.</t>
+  </si>
+  <si>
+    <t>1. Open Chrome Browser.
+2. Open https://shivohamautomation.com/.
+3. Scroll down to the "Course Categories" section.
+4. Observe the API Testing course card.
+5. Click the API Testing course card.</t>
+  </si>
+  <si>
+    <t>The user was redirected to the API Testing course page successfully and the page  displayed 3 courses, matching the count shown on the course card.</t>
+  </si>
+  <si>
+    <t>The user should be redirected to the API Testing course page, and the page should display 3 courses, matching the count shown on the course card.</t>
+  </si>
+  <si>
+    <t>TC_032</t>
+  </si>
+  <si>
+    <t>TC_033</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -462,6 +913,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -471,7 +928,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -494,17 +951,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -521,19 +1010,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -849,43 +1357,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70C44D14-D47B-40E2-B913-088EBF80304A}">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="85.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.88671875" customWidth="1"/>
-    <col min="7" max="7" width="36.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.109375" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" style="10" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="69" style="4" customWidth="1"/>
+    <col min="6" max="6" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.21875" customWidth="1"/>
+    <col min="8" max="8" width="37.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:10" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="11" t="s">
@@ -895,278 +1404,976 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="13">
+    <row r="2" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="13"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6" t="s">
+      <c r="I2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="12"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="13"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6" t="s">
+      <c r="I3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6" t="s">
+      <c r="I4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" ht="114" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="13"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6" t="s">
+      <c r="I5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" ht="122.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="I6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="12"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="I7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="12"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="7" t="s">
+    <row r="9" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="12"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="I9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="7" t="s">
+    <row r="11" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E22" s="3"/>
+    <row r="12" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="12">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="12"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="I16" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="12"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="12"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I19" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7">
+        <v>3</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="I24" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="I25" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="I26" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="I27" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="19">
+        <v>4</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G28" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="I28" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="20"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="H29" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="I29" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="12">
+        <v>5</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="I30" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="12"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="I31" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="12"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="I32" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="12"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="I33" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="12"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="I34" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D39" s="4"/>
+      <c r="E39"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D40" s="4"/>
+      <c r="E40"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D41" s="4"/>
+      <c r="E41"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D42" s="4"/>
+      <c r="E42"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D43" s="4"/>
+      <c r="E43"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D44" s="4"/>
+      <c r="E44"/>
+    </row>
+    <row r="61" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D61"/>
     </row>
     <row r="62" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D62"/>
@@ -1186,14 +2393,20 @@
     <row r="67" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D67"/>
     </row>
-    <row r="68" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D68"/>
-    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="10">
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B12:B19"/>
+    <mergeCell ref="A12:A19"/>
     <mergeCell ref="B2:B11"/>
     <mergeCell ref="A2:A11"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>